<commit_message>
Restore N/A in Manufacturer and Supplier seed lists; record decisions
Seed version bumped to v0-seed-3. The consistency test no longer allows
the N/A difference. PLAN.md records tonight's decisions and gets a
Progress log section.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/bioa/lookup_lists.xlsx
+++ b/clients/bioa/lookup_lists.xlsx
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A255"/>
+  <dimension ref="A1:A256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1851,693 +1851,700 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="4" t="inlineStr">
-        <is>
-          <t>NetSuite</t>
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>Neurogene Inc.</t>
+          <t>NetSuite</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>New England BioLabs</t>
+          <t>Neurogene Inc.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>Nikon</t>
+          <t>New England BioLabs</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>NuAire</t>
+          <t>Nikon</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Oakton</t>
+          <t>NuAire</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>OHAUS Corporation</t>
+          <t>Oakton</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>Olink Proteomics</t>
+          <t>OHAUS Corporation</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>Olympian</t>
+          <t>Olink Proteomics</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Olympian</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>Omni Inc.</t>
+          <t>Olympus</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>Omni Inc.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>Oxis Insrtuments Inc.</t>
+          <t>Oxford</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>PALL Scientific</t>
+          <t>Oxis Insrtuments Inc.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>PALL Scientific</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>Perkin Elmer</t>
+          <t>Panasonic</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>Phenix</t>
+          <t>Perkin Elmer</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>Plas Labs</t>
+          <t>Phenix</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>Polyfoam Packers Corp</t>
+          <t>Plas Labs</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Polymedco</t>
+          <t>Polyfoam Packers Corp</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Precision</t>
+          <t>Polymedco</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>Precision Systems Inc</t>
+          <t>Precision</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>Prices Scientific</t>
+          <t>Precision Systems Inc</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>Progen</t>
+          <t>Prices Scientific</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>Promega</t>
+          <t>Progen</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>ProPette</t>
+          <t>Promega</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>Protein Simple</t>
+          <t>ProPette</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>Pure Aire</t>
+          <t>Protein Simple</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>Qiagen</t>
+          <t>Pure Aire</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Qsonica</t>
+          <t>Qiagen</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>Quality Biological</t>
+          <t>Qsonica</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>Quanterix</t>
+          <t>Quality Biological</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>R and D Systems</t>
+          <t>Quanterix</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>Rainin</t>
+          <t>R and D Systems</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>Rees Scientific Corp</t>
+          <t>Rainin</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>Repligen</t>
+          <t>Rees Scientific Corp</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>Revco / Puffer Hubbard</t>
+          <t>Repligen</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>Revco / Puffer Hubbard</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Revvity</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>RoxyM Bel-Art</t>
+          <t>Roche</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>Sakura Finetek</t>
+          <t>RoxyM Bel-Art</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>Sanyo</t>
+          <t>Sakura Finetek</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>Sartorius</t>
+          <t>Sanyo</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>SAS</t>
+          <t>Sartorius</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>Savant</t>
+          <t>SAS</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>Scientific Industries</t>
+          <t>Savant</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>Scientific Products</t>
+          <t>Scientific Industries</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>Sciex</t>
+          <t>Scientific Products</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>Scinomix</t>
+          <t>Sciex</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>Scotsman</t>
+          <t>Scinomix</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>Security System</t>
+          <t>Scotsman</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>Shel Lab</t>
+          <t>Security System</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>Sheldon</t>
+          <t>Shel Lab</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Sheldon</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>Sigma</t>
+          <t>Siemens</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>SignaGen</t>
+          <t>Sigma</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>SolarWinds</t>
+          <t>SignaGen</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>Sorvall</t>
+          <t>SolarWinds</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>Stegmann Systems</t>
+          <t>Sorvall</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>StemCell Technologies</t>
+          <t>Stegmann Systems</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>Stirling</t>
+          <t>StemCell Technologies</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>Stratec Biomedical (Aesku)</t>
+          <t>Stirling</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>Symphony</t>
+          <t>Stratec Biomedical (Aesku)</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>Talboys</t>
+          <t>Symphony</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>Tecan</t>
+          <t>Talboys</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>Teknova</t>
+          <t>Tecan</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>Thermo Fisher</t>
+          <t>Teknova</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>Thermo Fisher Scientific</t>
+          <t>Thermo Fisher</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>ThermoFisher</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>Thermolyne</t>
+          <t>ThermoFisher</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>TMYTest</t>
+          <t>Thermolyne</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>Tomy</t>
+          <t>TMYTest</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>Traceable</t>
+          <t>Tomy</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>Transcat</t>
+          <t>Traceable</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>Troemner</t>
+          <t>Transcat</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>Troemner</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>Turbo Air</t>
+          <t>TTE</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>Tuttnauer</t>
+          <t>Turbo Air</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>Unchained Labs</t>
+          <t>Tuttnauer</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>Union Scientific Corporation</t>
+          <t>Unchained Labs</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>USA Scientific</t>
+          <t>Union Scientific Corporation</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>VistaLab</t>
+          <t>USA Scientific</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>Vistavision</t>
+          <t>VistaLab</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>VWR</t>
+          <t>Vistavision</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>VWR (Henry Troemner LLC)</t>
+          <t>VWR</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>VWR (Thermo Fisher Scientific)</t>
+          <t>VWR (Henry Troemner LLC)</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>VWR (True)</t>
+          <t>VWR (Thermo Fisher Scientific)</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>VWR (Visalia)</t>
+          <t>VWR (True)</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>Waters</t>
+          <t>VWR (Visalia)</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>Welch Manufacturing</t>
+          <t>Waters</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>Werther International</t>
+          <t>Welch Manufacturing</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>Woods</t>
+          <t>Werther International</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>Wuxi ATU</t>
+          <t>Woods</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>Wyatt Technology</t>
+          <t>Wuxi ATU</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>Zeiss</t>
+          <t>Wyatt Technology</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>Zeiss Axiovert</t>
+          <t>Zeiss</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>ZenQMS</t>
+          <t>Zeiss Axiovert</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>Ziath</t>
+          <t>ZenQMS</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>Ziath</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="4" t="inlineStr">
         <is>
           <t>Zymo Research</t>
         </is>
@@ -2693,7 +2700,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>v0-seed-2</t>
+          <t>v0-seed-3</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2720,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A255"/>
+  <dimension ref="A1:A256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -5225,693 +5232,700 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="4" t="inlineStr">
-        <is>
-          <t>NetSuite</t>
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>Neurogene Inc.</t>
+          <t>NetSuite</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>New England BioLabs</t>
+          <t>Neurogene Inc.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>Nikon</t>
+          <t>New England BioLabs</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>NuAire</t>
+          <t>Nikon</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>Oakton</t>
+          <t>NuAire</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>OHAUS Corporation</t>
+          <t>Oakton</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>Olink Proteomics</t>
+          <t>OHAUS Corporation</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>Olympian</t>
+          <t>Olink Proteomics</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>Olympus</t>
+          <t>Olympian</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>Omni Inc.</t>
+          <t>Olympus</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>Oxford</t>
+          <t>Omni Inc.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>Oxis Insrtuments Inc.</t>
+          <t>Oxford</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>PALL Scientific</t>
+          <t>Oxis Insrtuments Inc.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>PALL Scientific</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>Perkin Elmer</t>
+          <t>Panasonic</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>Phenix</t>
+          <t>Perkin Elmer</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>Plas Labs</t>
+          <t>Phenix</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>Polyfoam Packers Corp</t>
+          <t>Plas Labs</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Polymedco</t>
+          <t>Polyfoam Packers Corp</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>Precision</t>
+          <t>Polymedco</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>Precision Systems Inc</t>
+          <t>Precision</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>Prices Scientific</t>
+          <t>Precision Systems Inc</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>Progen</t>
+          <t>Prices Scientific</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>Promega</t>
+          <t>Progen</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>ProPette</t>
+          <t>Promega</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>Protein Simple</t>
+          <t>ProPette</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>Pure Aire</t>
+          <t>Protein Simple</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>Qiagen</t>
+          <t>Pure Aire</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>Qsonica</t>
+          <t>Qiagen</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>Quality Biological</t>
+          <t>Qsonica</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>Quanterix</t>
+          <t>Quality Biological</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>R and D Systems</t>
+          <t>Quanterix</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>Rainin</t>
+          <t>R and D Systems</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>Rees Scientific Corp</t>
+          <t>Rainin</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>Repligen</t>
+          <t>Rees Scientific Corp</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>Revco / Puffer Hubbard</t>
+          <t>Repligen</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>Revvity</t>
+          <t>Revco / Puffer Hubbard</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Revvity</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>RoxyM Bel-Art</t>
+          <t>Roche</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>Sakura Finetek</t>
+          <t>RoxyM Bel-Art</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>Sanyo</t>
+          <t>Sakura Finetek</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>Sartorius</t>
+          <t>Sanyo</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>SAS</t>
+          <t>Sartorius</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>Savant</t>
+          <t>SAS</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>Scientific Industries</t>
+          <t>Savant</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>Scientific Products</t>
+          <t>Scientific Industries</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>Sciex</t>
+          <t>Scientific Products</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>Scinomix</t>
+          <t>Sciex</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>Scotsman</t>
+          <t>Scinomix</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>Security System</t>
+          <t>Scotsman</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>Shel Lab</t>
+          <t>Security System</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>Sheldon</t>
+          <t>Shel Lab</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Sheldon</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>Sigma</t>
+          <t>Siemens</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>SignaGen</t>
+          <t>Sigma</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>SolarWinds</t>
+          <t>SignaGen</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>Sorvall</t>
+          <t>SolarWinds</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>Stegmann Systems</t>
+          <t>Sorvall</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>StemCell Technologies</t>
+          <t>Stegmann Systems</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>Stirling</t>
+          <t>StemCell Technologies</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>Stratec Biomedical (Aesku)</t>
+          <t>Stirling</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>Symphony</t>
+          <t>Stratec Biomedical (Aesku)</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>Talboys</t>
+          <t>Symphony</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>Tecan</t>
+          <t>Talboys</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>Teknova</t>
+          <t>Tecan</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>Thermo Fisher</t>
+          <t>Teknova</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>Thermo Fisher Scientific</t>
+          <t>Thermo Fisher</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>ThermoFisher</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>Thermolyne</t>
+          <t>ThermoFisher</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>TMYTest</t>
+          <t>Thermolyne</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>Tomy</t>
+          <t>TMYTest</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>Traceable</t>
+          <t>Tomy</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>Transcat</t>
+          <t>Traceable</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>Troemner</t>
+          <t>Transcat</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>Troemner</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>Turbo Air</t>
+          <t>TTE</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>Tuttnauer</t>
+          <t>Turbo Air</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>Unchained Labs</t>
+          <t>Tuttnauer</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>Union Scientific Corporation</t>
+          <t>Unchained Labs</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>USA Scientific</t>
+          <t>Union Scientific Corporation</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>VistaLab</t>
+          <t>USA Scientific</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>Vistavision</t>
+          <t>VistaLab</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>VWR</t>
+          <t>Vistavision</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>VWR (Henry Troemner LLC)</t>
+          <t>VWR</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>VWR (Thermo Fisher Scientific)</t>
+          <t>VWR (Henry Troemner LLC)</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>VWR (True)</t>
+          <t>VWR (Thermo Fisher Scientific)</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>VWR (Visalia)</t>
+          <t>VWR (True)</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>Waters</t>
+          <t>VWR (Visalia)</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>Welch Manufacturing</t>
+          <t>Waters</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>Werther International</t>
+          <t>Welch Manufacturing</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>Woods</t>
+          <t>Werther International</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>Wuxi ATU</t>
+          <t>Woods</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>Wyatt Technology</t>
+          <t>Wuxi ATU</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>Zeiss</t>
+          <t>Wyatt Technology</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>Zeiss Axiovert</t>
+          <t>Zeiss</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>ZenQMS</t>
+          <t>Zeiss Axiovert</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>Ziath</t>
+          <t>ZenQMS</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>Ziath</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="4" t="inlineStr">
         <is>
           <t>Zymo Research</t>
         </is>

</xml_diff>